<commit_message>
chore: refresh plotly embeds from source repo
</commit_message>
<xml_diff>
--- a/embeds/data/economy-living-standards/slot-13-소득분위별-월평균-소비지출액과-소비지출비,-2024.xlsx
+++ b/embeds/data/economy-living-standards/slot-13-소득분위별-월평균-소비지출액과-소비지출비,-2024.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>소비지출액(만 원)</t>
+          <t>소비지출액</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -484,7 +484,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>소비지출액(만 원)</t>
+          <t>소비지출액</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>소비지출액(만 원)</t>
+          <t>소비지출액</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -530,7 +530,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>소비지출액(만 원)</t>
+          <t>소비지출액</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>소비지출액(만 원)</t>
+          <t>소비지출액</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -576,7 +576,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>소비지출비(%)</t>
+          <t>소비지출비</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>소비지출비(%)</t>
+          <t>소비지출비</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -622,7 +622,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>소비지출비(%)</t>
+          <t>소비지출비</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -645,7 +645,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>소비지출비(%)</t>
+          <t>소비지출비</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>소비지출비(%)</t>
+          <t>소비지출비</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>